<commit_message>
Add Navy FY27 budget books; checkpoint cross-project WIP
budget_books: download_navy_books.py + _manifest_navy_fy27.csv pull the full
FY27 (PB-2027) Department of the Navy justification set (APN/WPN/PANMC/SCN/OPN/
PMC, RDTEN, OMN+reserve/USMC, MilPers, MCON, NWCF, Highlights). The large book
PDFs/txt are gitignored (book binaries stay local; the script + manifest make
the corpus reproducible).

Also folds in working-tree WIP across projects:
- awards_methodology: deck slide restructure (two-routes/prime/subcontractor
  specs, slides_new, archive), recompete methodology + playbook, Saronic
  navy-widened contract research pulls.
- distributed_shipbuilding: TAM/SAM workbook refresh, deck logs,
  ddg_module_cost, deck_data_reference.
- style_library: library.pptx + bulk-conversion / table-kit refactor logs.
- deck_core: slide_probe reports; primitives.py tweak.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/distributed_shipbuilding/tam/master/20260620_Distributed Shipbuilding Master TAM_vS.xlsx
+++ b/projects/distributed_shipbuilding/tam/master/20260620_Distributed Shipbuilding Master TAM_vS.xlsx
@@ -51,37 +51,11 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">HII FY2026 target: outsourcing hours +30% y/y.</t>
+          <t xml:space="preserve">HII FY2026 target: outsourcing hours +30% y/y. Phased onto the outyear BC coefficient as a compound ramp reaching the full +30% at FY2031 (no throughput normalization).</t>
         </r>
       </text>
     </comment>
     <comment ref="C25" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">HII FY2026 target: shipbuilding throughput +15%.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C26" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Intensity growth = 1.30 / 1.15 - 1 = 13.0%; applied once.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C27" authorId="0">
       <text>
         <r>
           <rPr>
@@ -351,7 +325,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -434,6 +408,14 @@
     <xf numFmtId="169" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="169" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
@@ -443,8 +425,36 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="6">
     <dxf/>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE2EFDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -539,7 +549,7 @@
       <c r="I2" s="8"/>
     </row>
     <row r="3" outlineLevel="1">
-      <c r="B3" s="56" t="inlineStr">
+      <c r="B3" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">Portfolio outsourced TAM, FY2022-31, constant FY2026 $M</t>
         </is>
@@ -790,7 +800,7 @@
       <c r="I20" s="16"/>
     </row>
     <row r="21" outlineLevel="2">
-      <c r="B21" s="56" t="inlineStr">
+      <c r="B21" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">E = estimate: FY2026-27 budget request (FY2026 incl. OBBBA).</t>
         </is>
@@ -995,9 +1005,9 @@
       </c>
     </row>
     <row r="35" outlineLevel="2">
-      <c r="B35" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Low holds coefficients flat; high applies Assumptions §4.</t>
+      <c r="B35" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low holds coefficients flat; high compound-ramps Assumptions §4 growth to FY2031.</t>
         </is>
       </c>
     </row>
@@ -1045,7 +1055,7 @@
       <c r="I2" s="8"/>
     </row>
     <row r="3" outlineLevel="1">
-      <c r="B3" s="56" t="inlineStr">
+      <c r="B3" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">PB2027 P-40 gross spend, FY2025-31</t>
         </is>
@@ -1701,25 +1711,25 @@
           <t xml:space="preserve">Constant-FY2026 factor (then-year x this; from Deflators)</t>
         </is>
       </c>
-      <c r="C41" s="57">
+      <c r="C41" s="61">
         <f>'Deflators'!D12</f>
       </c>
-      <c r="D41" s="57">
+      <c r="D41" s="61">
         <f>'Deflators'!D13</f>
       </c>
-      <c r="E41" s="57">
+      <c r="E41" s="61">
         <f>'Deflators'!D14</f>
       </c>
-      <c r="F41" s="57">
+      <c r="F41" s="61">
         <f>'Deflators'!D15</f>
       </c>
-      <c r="G41" s="57">
+      <c r="G41" s="61">
         <f>'Deflators'!D16</f>
       </c>
-      <c r="H41" s="57">
+      <c r="H41" s="61">
         <f>'Deflators'!D17</f>
       </c>
-      <c r="I41" s="57">
+      <c r="I41" s="61">
         <f>'Deflators'!D18</f>
       </c>
     </row>
@@ -1871,7 +1881,7 @@
       <c r="E2" s="8"/>
     </row>
     <row r="3" outlineLevel="1">
-      <c r="B3" s="56" t="inlineStr">
+      <c r="B3" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">Procurement deflators rebased to FY2026</t>
         </is>
@@ -1926,7 +1936,7 @@
       <c r="C9" s="5">
         <v>93.13</v>
       </c>
-      <c r="D9" s="57">
+      <c r="D9" s="61">
         <v>1.1</v>
       </c>
       <c r="E9" s="0" t="inlineStr">
@@ -1944,7 +1954,7 @@
       <c r="C10" s="5">
         <v>95.77</v>
       </c>
-      <c r="D10" s="57">
+      <c r="D10" s="61">
         <v>1.07</v>
       </c>
       <c r="E10" s="0" t="inlineStr">
@@ -1962,7 +1972,7 @@
       <c r="C11" s="5">
         <v>97.92</v>
       </c>
-      <c r="D11" s="57">
+      <c r="D11" s="61">
         <v>1.04</v>
       </c>
       <c r="E11" s="0" t="inlineStr">
@@ -1980,7 +1990,7 @@
       <c r="C12" s="5">
         <v>100.0</v>
       </c>
-      <c r="D12" s="57">
+      <c r="D12" s="61">
         <v>1.02</v>
       </c>
       <c r="E12" s="0" t="inlineStr">
@@ -1998,7 +2008,7 @@
       <c r="C13" s="5">
         <v>102.1</v>
       </c>
-      <c r="D13" s="57">
+      <c r="D13" s="61">
         <v>1.0</v>
       </c>
       <c r="E13" s="0" t="inlineStr">
@@ -2016,7 +2026,7 @@
       <c r="C14" s="5">
         <v>104.24</v>
       </c>
-      <c r="D14" s="57">
+      <c r="D14" s="61">
         <v>0.98</v>
       </c>
       <c r="E14" s="0" t="inlineStr">
@@ -2034,7 +2044,7 @@
       <c r="C15" s="5">
         <v>106.43</v>
       </c>
-      <c r="D15" s="57">
+      <c r="D15" s="61">
         <v>0.96</v>
       </c>
       <c r="E15" s="0" t="inlineStr">
@@ -2052,7 +2062,7 @@
       <c r="C16" s="5">
         <v>108.67</v>
       </c>
-      <c r="D16" s="57">
+      <c r="D16" s="61">
         <v>0.94</v>
       </c>
       <c r="E16" s="0" t="inlineStr">
@@ -2070,7 +2080,7 @@
       <c r="C17" s="5">
         <v>110.95</v>
       </c>
-      <c r="D17" s="57">
+      <c r="D17" s="61">
         <v>0.92</v>
       </c>
       <c r="E17" s="0" t="inlineStr">
@@ -2088,7 +2098,7 @@
       <c r="C18" s="5">
         <v>113.28</v>
       </c>
-      <c r="D18" s="57">
+      <c r="D18" s="61">
         <v>0.9</v>
       </c>
       <c r="E18" s="0" t="inlineStr">
@@ -2185,7 +2195,7 @@
       <c r="D2" s="8"/>
     </row>
     <row r="3" outlineLevel="1">
-      <c r="B3" s="56" t="inlineStr">
+      <c r="B3" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">Input bounds, outyear ordering, and completeness</t>
         </is>
@@ -2417,7 +2427,7 @@
         </is>
       </c>
       <c r="C28" s="44">
-        <f>COUNT('Assumptions'!C9,'Assumptions'!C18,'Assumptions'!C26,'Assumptions'!C27,'Assumptions'!E15,'Assumptions'!E16)</f>
+        <f>COUNT('Assumptions'!C9,'Assumptions'!C18,'Assumptions'!C24,'Assumptions'!C25,'Assumptions'!E15,'Assumptions'!E16)</f>
       </c>
       <c r="D28" s="0">
         <f>IF(C28=6,"OK","FAIL")</f>
@@ -2455,10 +2465,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D9:D28 D33">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
       <formula>"FAIL"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="2" operator="equal">
       <formula>"CHECK FAILED"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2493,7 +2503,7 @@
       <c r="C2" s="8"/>
     </row>
     <row r="3" outlineLevel="1">
-      <c r="B3" s="56" t="inlineStr">
+      <c r="B3" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">TAM definition, formula, scope, coefficient basis, and sources</t>
         </is>
@@ -2840,7 +2850,7 @@
       <c r="H2" s="8"/>
     </row>
     <row r="3" outlineLevel="1">
-      <c r="B3" s="56" t="inlineStr">
+      <c r="B3" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">Editable supplier-share, OBBBA, and outyear assumptions</t>
         </is>
@@ -2885,7 +2895,7 @@
           <t xml:space="preserve">DDG AP/LLTM supplier coefficient</t>
         </is>
       </c>
-      <c r="C9" s="59">
+      <c r="C9" s="63">
         <v>1.0</v>
       </c>
     </row>
@@ -2941,7 +2951,7 @@
       <c r="C15" s="12">
         <f>'SCN Budget'!G34</f>
       </c>
-      <c r="D15" s="59">
+      <c r="D15" s="63">
         <v>0</v>
       </c>
       <c r="E15" s="6">
@@ -2954,10 +2964,10 @@
           <t xml:space="preserve">DDG-51 OBBBA BC share (Sec. 20002(17))</t>
         </is>
       </c>
-      <c r="C16" s="59">
+      <c r="C16" s="63">
         <v>0.628</v>
       </c>
-      <c r="D16" s="59">
+      <c r="D16" s="63">
         <v>0</v>
       </c>
       <c r="E16" s="6">
@@ -2971,7 +2981,7 @@
           <t xml:space="preserve">FY2027 execution spillover</t>
         </is>
       </c>
-      <c r="C18" s="59">
+      <c r="C18" s="63">
         <v>0</v>
       </c>
     </row>
@@ -2985,7 +2995,7 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">§4 - Outyear intensity growth</t>
+          <t xml:space="preserve">§4 - Outyear outsourcing growth</t>
         </is>
       </c>
       <c r="C21" s="9"/>
@@ -3011,40 +3021,20 @@
     <row r="24" outlineLevel="2">
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">HII outsourcing-hours growth</t>
-        </is>
-      </c>
-      <c r="C24" s="59">
+          <t xml:space="preserve">HII outsourcing-hours growth (annual)</t>
+        </is>
+      </c>
+      <c r="C24" s="63">
         <v>0.3</v>
       </c>
     </row>
     <row r="25" outlineLevel="2">
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">HII shipbuilding-throughput growth</t>
-        </is>
-      </c>
-      <c r="C25" s="59">
-        <v>0.15</v>
-      </c>
-    </row>
-    <row r="26" outlineLevel="2">
-      <c r="B26" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Outsourcing intensity growth</t>
-        </is>
-      </c>
-      <c r="C26" s="6">
-        <f>(1+C24)/(1+C25)-1</f>
-      </c>
-    </row>
-    <row r="27" outlineLevel="2">
-      <c r="B27" s="0" t="inlineStr">
-        <is>
           <t xml:space="preserve">DDG-51 HII share of BC</t>
         </is>
       </c>
-      <c r="C27" s="59">
+      <c r="C25" s="63">
         <v>0.55</v>
       </c>
     </row>
@@ -3093,7 +3083,7 @@
       <c r="I2" s="8"/>
     </row>
     <row r="3" outlineLevel="1">
-      <c r="B3" s="56" t="inlineStr">
+      <c r="B3" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">Virginia BC and OBBBA TAM, FY2022-31</t>
         </is>
@@ -3726,87 +3716,96 @@
     <row r="50" outlineLevel="2">
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Outsourcing intensity growth</t>
+          <t xml:space="preserve">Outyear outsourcing growth (annual target)</t>
         </is>
       </c>
       <c r="C50" s="12">
-        <f>'Assumptions'!C26</f>
-      </c>
-    </row>
-    <row r="51" outlineLevel="2">
-      <c r="B51" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Outyear BC coefficient, high</t>
-        </is>
-      </c>
-      <c r="C51" s="6">
-        <f>C49*(1+C50)</f>
-      </c>
-    </row>
-    <row r="52" outlineLevel="2"/>
+        <f>'Assumptions'!C24</f>
+      </c>
+    </row>
+    <row r="51" outlineLevel="2"/>
+    <row r="52" outlineLevel="2">
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Outyears</t>
+        </is>
+      </c>
+      <c r="C52" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FY2028</t>
+        </is>
+      </c>
+      <c r="D52" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FY2029</t>
+        </is>
+      </c>
+      <c r="E52" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FY2030</t>
+        </is>
+      </c>
+      <c r="F52" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FY2031</t>
+        </is>
+      </c>
+    </row>
     <row r="53" outlineLevel="2">
-      <c r="B53" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Outyear ($M)</t>
-        </is>
-      </c>
-      <c r="C53" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FY2028</t>
-        </is>
-      </c>
-      <c r="D53" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FY2029</t>
-        </is>
-      </c>
-      <c r="E53" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FY2030</t>
-        </is>
-      </c>
-      <c r="F53" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FY2031</t>
-        </is>
+      <c r="B53" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FYDP gross</t>
+        </is>
+      </c>
+      <c r="C53" s="11">
+        <f>'FYDP Outyears'!F42</f>
+      </c>
+      <c r="D53" s="11">
+        <f>'FYDP Outyears'!G42</f>
+      </c>
+      <c r="E53" s="11">
+        <f>'FYDP Outyears'!H42</f>
+      </c>
+      <c r="F53" s="11">
+        <f>'FYDP Outyears'!I42</f>
       </c>
     </row>
     <row r="54" outlineLevel="2">
-      <c r="B54" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FYDP gross</t>
-        </is>
-      </c>
-      <c r="C54" s="11">
-        <f>'FYDP Outyears'!F42</f>
-      </c>
-      <c r="D54" s="11">
-        <f>'FYDP Outyears'!G42</f>
-      </c>
-      <c r="E54" s="11">
-        <f>'FYDP Outyears'!H42</f>
-      </c>
-      <c r="F54" s="11">
-        <f>'FYDP Outyears'!I42</f>
+      <c r="B54" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Outyear BC base</t>
+        </is>
+      </c>
+      <c r="C54" s="4">
+        <f>C53*$C$48</f>
+      </c>
+      <c r="D54" s="4">
+        <f>D53*$C$48</f>
+      </c>
+      <c r="E54" s="4">
+        <f>E53*$C$48</f>
+      </c>
+      <c r="F54" s="4">
+        <f>F53*$C$48</f>
       </c>
     </row>
     <row r="55" outlineLevel="2">
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Outyear BC base</t>
-        </is>
-      </c>
-      <c r="C55" s="4">
-        <f>C54*$C$48</f>
-      </c>
-      <c r="D55" s="4">
-        <f>D54*$C$48</f>
-      </c>
-      <c r="E55" s="4">
-        <f>E54*$C$48</f>
-      </c>
-      <c r="F55" s="4">
-        <f>F54*$C$48</f>
+          <t xml:space="preserve">Outyear BC coefficient, high (compounded)</t>
+        </is>
+      </c>
+      <c r="C55" s="6">
+        <f>$C$49*POWER(1+$C$50,1/4)</f>
+      </c>
+      <c r="D55" s="6">
+        <f>$C$49*POWER(1+$C$50,2/4)</f>
+      </c>
+      <c r="E55" s="6">
+        <f>$C$49*POWER(1+$C$50,3/4)</f>
+      </c>
+      <c r="F55" s="6">
+        <f>$C$49*POWER(1+$C$50,4/4)</f>
       </c>
     </row>
     <row r="56" outlineLevel="2">
@@ -3816,16 +3815,16 @@
         </is>
       </c>
       <c r="C56" s="4">
-        <f>C55*$C$49</f>
+        <f>C54*$C$49</f>
       </c>
       <c r="D56" s="4">
-        <f>D55*$C$49</f>
+        <f>D54*$C$49</f>
       </c>
       <c r="E56" s="4">
-        <f>E55*$C$49</f>
+        <f>E54*$C$49</f>
       </c>
       <c r="F56" s="4">
-        <f>F55*$C$49</f>
+        <f>F54*$C$49</f>
       </c>
     </row>
     <row r="57" outlineLevel="2">
@@ -3835,16 +3834,16 @@
         </is>
       </c>
       <c r="C57" s="4">
-        <f>C55*$C$51</f>
+        <f>C54*C55</f>
       </c>
       <c r="D57" s="4">
-        <f>D55*$C$51</f>
+        <f>D54*D55</f>
       </c>
       <c r="E57" s="4">
-        <f>E55*$C$51</f>
+        <f>E54*E55</f>
       </c>
       <c r="F57" s="4">
-        <f>F55*$C$51</f>
+        <f>F54*F55</f>
       </c>
     </row>
     <row r="58" outlineLevel="2"/>
@@ -3912,7 +3911,7 @@
       <c r="I2" s="8"/>
     </row>
     <row r="3" outlineLevel="1">
-      <c r="B3" s="56" t="inlineStr">
+      <c r="B3" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">Columbia BC TAM, FY2022-31</t>
         </is>
@@ -4444,87 +4443,96 @@
     <row r="45" outlineLevel="2">
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Outsourcing intensity growth</t>
+          <t xml:space="preserve">Outyear outsourcing growth (annual target)</t>
         </is>
       </c>
       <c r="C45" s="12">
-        <f>'Assumptions'!C26</f>
-      </c>
-    </row>
-    <row r="46" outlineLevel="2">
-      <c r="B46" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Outyear BC coefficient, high</t>
-        </is>
-      </c>
-      <c r="C46" s="6">
-        <f>C44*(1+C45)</f>
-      </c>
-    </row>
-    <row r="47" outlineLevel="2"/>
+        <f>'Assumptions'!C24</f>
+      </c>
+    </row>
+    <row r="46" outlineLevel="2"/>
+    <row r="47" outlineLevel="2">
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Outyears</t>
+        </is>
+      </c>
+      <c r="C47" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FY2028</t>
+        </is>
+      </c>
+      <c r="D47" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FY2029</t>
+        </is>
+      </c>
+      <c r="E47" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FY2030</t>
+        </is>
+      </c>
+      <c r="F47" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FY2031</t>
+        </is>
+      </c>
+    </row>
     <row r="48" outlineLevel="2">
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Outyear ($M)</t>
-        </is>
-      </c>
-      <c r="C48" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FY2028</t>
-        </is>
-      </c>
-      <c r="D48" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FY2029</t>
-        </is>
-      </c>
-      <c r="E48" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FY2030</t>
-        </is>
-      </c>
-      <c r="F48" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FY2031</t>
-        </is>
+      <c r="B48" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FYDP gross</t>
+        </is>
+      </c>
+      <c r="C48" s="11">
+        <f>'FYDP Outyears'!F43</f>
+      </c>
+      <c r="D48" s="11">
+        <f>'FYDP Outyears'!G43</f>
+      </c>
+      <c r="E48" s="11">
+        <f>'FYDP Outyears'!H43</f>
+      </c>
+      <c r="F48" s="11">
+        <f>'FYDP Outyears'!I43</f>
       </c>
     </row>
     <row r="49" outlineLevel="2">
-      <c r="B49" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FYDP gross</t>
-        </is>
-      </c>
-      <c r="C49" s="11">
-        <f>'FYDP Outyears'!F43</f>
-      </c>
-      <c r="D49" s="11">
-        <f>'FYDP Outyears'!G43</f>
-      </c>
-      <c r="E49" s="11">
-        <f>'FYDP Outyears'!H43</f>
-      </c>
-      <c r="F49" s="11">
-        <f>'FYDP Outyears'!I43</f>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Outyear BC base</t>
+        </is>
+      </c>
+      <c r="C49" s="4">
+        <f>C48*$C$43</f>
+      </c>
+      <c r="D49" s="4">
+        <f>D48*$C$43</f>
+      </c>
+      <c r="E49" s="4">
+        <f>E48*$C$43</f>
+      </c>
+      <c r="F49" s="4">
+        <f>F48*$C$43</f>
       </c>
     </row>
     <row r="50" outlineLevel="2">
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Outyear BC base</t>
-        </is>
-      </c>
-      <c r="C50" s="4">
-        <f>C49*$C$43</f>
-      </c>
-      <c r="D50" s="4">
-        <f>D49*$C$43</f>
-      </c>
-      <c r="E50" s="4">
-        <f>E49*$C$43</f>
-      </c>
-      <c r="F50" s="4">
-        <f>F49*$C$43</f>
+          <t xml:space="preserve">Outyear BC coefficient, high (compounded)</t>
+        </is>
+      </c>
+      <c r="C50" s="6">
+        <f>$C$44*POWER(1+$C$45,1/4)</f>
+      </c>
+      <c r="D50" s="6">
+        <f>$C$44*POWER(1+$C$45,2/4)</f>
+      </c>
+      <c r="E50" s="6">
+        <f>$C$44*POWER(1+$C$45,3/4)</f>
+      </c>
+      <c r="F50" s="6">
+        <f>$C$44*POWER(1+$C$45,4/4)</f>
       </c>
     </row>
     <row r="51" outlineLevel="2">
@@ -4534,16 +4542,16 @@
         </is>
       </c>
       <c r="C51" s="4">
-        <f>C50*$C$44</f>
+        <f>C49*$C$44</f>
       </c>
       <c r="D51" s="4">
-        <f>D50*$C$44</f>
+        <f>D49*$C$44</f>
       </c>
       <c r="E51" s="4">
-        <f>E50*$C$44</f>
+        <f>E49*$C$44</f>
       </c>
       <c r="F51" s="4">
-        <f>F50*$C$44</f>
+        <f>F49*$C$44</f>
       </c>
     </row>
     <row r="52" outlineLevel="2">
@@ -4553,16 +4561,16 @@
         </is>
       </c>
       <c r="C52" s="4">
-        <f>C50*$C$46</f>
+        <f>C49*C50</f>
       </c>
       <c r="D52" s="4">
-        <f>D50*$C$46</f>
+        <f>D49*D50</f>
       </c>
       <c r="E52" s="4">
-        <f>E50*$C$46</f>
+        <f>E49*E50</f>
       </c>
       <c r="F52" s="4">
-        <f>F50*$C$46</f>
+        <f>F49*F50</f>
       </c>
     </row>
     <row r="53" outlineLevel="2"/>
@@ -4630,7 +4638,7 @@
       <c r="I2" s="8"/>
     </row>
     <row r="3" outlineLevel="1">
-      <c r="B3" s="56" t="inlineStr">
+      <c r="B3" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">DDG-51 BC, AP/LLTM, and OBBBA TAM, FY2022-31</t>
         </is>
@@ -5349,11 +5357,11 @@
     <row r="55" outlineLevel="2">
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Outsourcing intensity growth</t>
+          <t xml:space="preserve">Outyear outsourcing growth (annual target)</t>
         </is>
       </c>
       <c r="C55" s="12">
-        <f>'Assumptions'!C26</f>
+        <f>'Assumptions'!C24</f>
       </c>
     </row>
     <row r="56" outlineLevel="2">
@@ -5363,83 +5371,92 @@
         </is>
       </c>
       <c r="C56" s="12">
-        <f>'Assumptions'!C27</f>
-      </c>
-    </row>
-    <row r="57" outlineLevel="2">
-      <c r="B57" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Outyear BC coefficient, high</t>
-        </is>
-      </c>
-      <c r="C57" s="6">
-        <f>C54*(1+C56*C55)</f>
-      </c>
-    </row>
-    <row r="58" outlineLevel="2"/>
+        <f>'Assumptions'!C25</f>
+      </c>
+    </row>
+    <row r="57" outlineLevel="2"/>
+    <row r="58" outlineLevel="2">
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Outyears</t>
+        </is>
+      </c>
+      <c r="C58" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FY2028</t>
+        </is>
+      </c>
+      <c r="D58" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FY2029</t>
+        </is>
+      </c>
+      <c r="E58" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FY2030</t>
+        </is>
+      </c>
+      <c r="F58" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FY2031</t>
+        </is>
+      </c>
+    </row>
     <row r="59" outlineLevel="2">
-      <c r="B59" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Outyear ($M)</t>
-        </is>
-      </c>
-      <c r="C59" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FY2028</t>
-        </is>
-      </c>
-      <c r="D59" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FY2029</t>
-        </is>
-      </c>
-      <c r="E59" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FY2030</t>
-        </is>
-      </c>
-      <c r="F59" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FY2031</t>
-        </is>
+      <c r="B59" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FYDP gross</t>
+        </is>
+      </c>
+      <c r="C59" s="11">
+        <f>'FYDP Outyears'!F44</f>
+      </c>
+      <c r="D59" s="11">
+        <f>'FYDP Outyears'!G44</f>
+      </c>
+      <c r="E59" s="11">
+        <f>'FYDP Outyears'!H44</f>
+      </c>
+      <c r="F59" s="11">
+        <f>'FYDP Outyears'!I44</f>
       </c>
     </row>
     <row r="60" outlineLevel="2">
-      <c r="B60" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FYDP gross</t>
-        </is>
-      </c>
-      <c r="C60" s="11">
-        <f>'FYDP Outyears'!F44</f>
-      </c>
-      <c r="D60" s="11">
-        <f>'FYDP Outyears'!G44</f>
-      </c>
-      <c r="E60" s="11">
-        <f>'FYDP Outyears'!H44</f>
-      </c>
-      <c r="F60" s="11">
-        <f>'FYDP Outyears'!I44</f>
+      <c r="B60" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Outyear BC base</t>
+        </is>
+      </c>
+      <c r="C60" s="4">
+        <f>C59*$C$53</f>
+      </c>
+      <c r="D60" s="4">
+        <f>D59*$C$53</f>
+      </c>
+      <c r="E60" s="4">
+        <f>E59*$C$53</f>
+      </c>
+      <c r="F60" s="4">
+        <f>F59*$C$53</f>
       </c>
     </row>
     <row r="61" outlineLevel="2">
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Outyear BC base</t>
-        </is>
-      </c>
-      <c r="C61" s="4">
-        <f>C60*$C$53</f>
-      </c>
-      <c r="D61" s="4">
-        <f>D60*$C$53</f>
-      </c>
-      <c r="E61" s="4">
-        <f>E60*$C$53</f>
-      </c>
-      <c r="F61" s="4">
-        <f>F60*$C$53</f>
+          <t xml:space="preserve">Outyear BC coefficient, high (compounded)</t>
+        </is>
+      </c>
+      <c r="C61" s="6">
+        <f>$C$54*(1+$C$56*(POWER(1+$C$55,1/4)-1))</f>
+      </c>
+      <c r="D61" s="6">
+        <f>$C$54*(1+$C$56*(POWER(1+$C$55,2/4)-1))</f>
+      </c>
+      <c r="E61" s="6">
+        <f>$C$54*(1+$C$56*(POWER(1+$C$55,3/4)-1))</f>
+      </c>
+      <c r="F61" s="6">
+        <f>$C$54*(1+$C$56*(POWER(1+$C$55,4/4)-1))</f>
       </c>
     </row>
     <row r="62" outlineLevel="2">
@@ -5449,16 +5466,16 @@
         </is>
       </c>
       <c r="C62" s="4">
-        <f>C61*$C$54</f>
+        <f>C60*$C$54</f>
       </c>
       <c r="D62" s="4">
-        <f>D61*$C$54</f>
+        <f>D60*$C$54</f>
       </c>
       <c r="E62" s="4">
-        <f>E61*$C$54</f>
+        <f>E60*$C$54</f>
       </c>
       <c r="F62" s="4">
-        <f>F61*$C$54</f>
+        <f>F60*$C$54</f>
       </c>
     </row>
     <row r="63" outlineLevel="2">
@@ -5468,16 +5485,16 @@
         </is>
       </c>
       <c r="C63" s="4">
-        <f>C61*$C$57</f>
+        <f>C60*C61</f>
       </c>
       <c r="D63" s="4">
-        <f>D61*$C$57</f>
+        <f>D60*D61</f>
       </c>
       <c r="E63" s="4">
-        <f>E61*$C$57</f>
+        <f>E60*E61</f>
       </c>
       <c r="F63" s="4">
-        <f>F61*$C$57</f>
+        <f>F60*F61</f>
       </c>
     </row>
     <row r="64" outlineLevel="2"/>
@@ -5545,7 +5562,7 @@
       <c r="I2" s="8"/>
     </row>
     <row r="3" outlineLevel="1">
-      <c r="B3" s="56" t="inlineStr">
+      <c r="B3" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">PB2027 P-5c cost categories and constant-dollar BC bases</t>
         </is>
@@ -5733,22 +5750,22 @@
           <t xml:space="preserve">Constant-FY2026 factor (then-year x this; from Deflators)</t>
         </is>
       </c>
-      <c r="C13" s="57">
+      <c r="C13" s="61">
         <f>'Deflators'!D9</f>
       </c>
-      <c r="D13" s="57">
+      <c r="D13" s="61">
         <f>'Deflators'!D10</f>
       </c>
-      <c r="E13" s="57">
+      <c r="E13" s="61">
         <f>'Deflators'!D11</f>
       </c>
-      <c r="F13" s="57">
+      <c r="F13" s="61">
         <f>'Deflators'!D12</f>
       </c>
-      <c r="G13" s="57">
+      <c r="G13" s="61">
         <f>'Deflators'!D13</f>
       </c>
-      <c r="H13" s="57">
+      <c r="H13" s="61">
         <f>'Deflators'!D14</f>
       </c>
     </row>
@@ -8075,7 +8092,7 @@
       <c r="O2" s="8"/>
     </row>
     <row r="3" outlineLevel="1">
-      <c r="B3" s="56" t="inlineStr">
+      <c r="B3" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">Award place of performance and supplier coefficients</t>
         </is>
@@ -11384,7 +11401,7 @@
       <c r="H2" s="8"/>
     </row>
     <row r="3" outlineLevel="1">
-      <c r="B3" s="56" t="inlineStr">
+      <c r="B3" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">FY2026 mandatory awards and BC/GFE bridge</t>
         </is>

</xml_diff>